<commit_message>
Phase 8 complétée : Nouveau système de mapping avec valeurs prédéfinies
- Step 8.1-8.6 : Backend - Table allowed_mappings, validation, dropdowns filtrés, recalcul automatique
- Step 8.7 : Frontend - Gestion table allowed_mappings avec création de nouvelles valeurs et reset
- Step 8.8 : Frontend - Fonctionnalité bouton ✏️ (déjà OK)
- Reset mappings autorisés : supprime mappings invalides et réinitialise transactions associées
- Tous les critères d'acceptation globaux Phase 8 remplis
</commit_message>
<xml_diff>
--- a/backend/data/input/trades/test_mappings.xlsx
+++ b/backend/data/input/trades/test_mappings.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,66 +453,110 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PRLV SEPA</t>
+          <t>TEST VALID 1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CHARGES</t>
+          <t>Adhésion Organisme de Gestion Agréé (OGA)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>FRAIS BANCAIRES</t>
+          <t>Autres dépenses</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>PRLV</t>
+          <t>Charges Déductibles</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VIR STRIPE</t>
+          <t>TEST VALID 2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PRODUITS</t>
+          <t>Adhésion Organisme de Gestion Agréé (OGA)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>REVENUS LOCATIFS</t>
+          <t>Autres dépenses</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>STRIPE</t>
+          <t>Charges Déductibles</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CARTE</t>
+          <t>TEST INVALID 1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CHARGES</t>
+          <t>INVALID_LEVEL1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>FRAIS BANCAIRES</t>
+          <t>INVALID_LEVEL2</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CARTE BLEUE</t>
+          <t>INVALID_LEVEL3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TEST INVALID 2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Adhésion Organisme de Gestion Agréé (OGA)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>INVALID_LEVEL2_COMBO</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>INVALID_LEVEL3_COMBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TEST VALID 3</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Adhésion Organisme de Gestion Agréé (OGA)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Autres dépenses</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Charges Déductibles</t>
         </is>
       </c>
     </row>

</xml_diff>